<commit_message>
Agrega el Simulador de escenarios y la versión 1.2 del prototipo
- Simulador: meta de rotación, costo supuesto por reemplazo, resultados, gráficos,
  comparación de hasta 3 escenarios y copia en CSV; respeta los filtros.
- Fórmulas centralizadas en calc.ts (simularEscenario, validarMeta, validarCosto).
- Mejoras de claridad: lectura ejecutiva, ranking de causas, plan de acción,
  semáforo explicado, glosario y seguimiento ampliado.
- 81 pruebas automatizadas aprobadas; documento de cierre actualizado.
</commit_message>
<xml_diff>
--- a/metricas/burndown/burndown_seguimiento.xlsx
+++ b/metricas/burndown/burndown_seguimiento.xlsx
@@ -828,11 +828,11 @@
           </c:spPr>
         </c:hiLowLines>
         <c:marker val="0"/>
-        <c:axId val="79916803"/>
-        <c:axId val="98896579"/>
+        <c:axId val="47667334"/>
+        <c:axId val="96684025"/>
       </c:lineChart>
       <c:catAx>
-        <c:axId val="79916803"/>
+        <c:axId val="47667334"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -898,7 +898,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="98896579"/>
+        <c:crossAx val="96684025"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -906,7 +906,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="98896579"/>
+        <c:axId val="96684025"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -982,7 +982,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="79916803"/>
+        <c:crossAx val="47667334"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -1219,11 +1219,11 @@
           </c:spPr>
         </c:hiLowLines>
         <c:marker val="0"/>
-        <c:axId val="42318755"/>
-        <c:axId val="55314174"/>
+        <c:axId val="25717858"/>
+        <c:axId val="11710884"/>
       </c:lineChart>
       <c:catAx>
-        <c:axId val="42318755"/>
+        <c:axId val="25717858"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -1289,7 +1289,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="55314174"/>
+        <c:crossAx val="11710884"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -1297,7 +1297,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="55314174"/>
+        <c:axId val="11710884"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -1373,7 +1373,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="42318755"/>
+        <c:crossAx val="25717858"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -1610,11 +1610,11 @@
           </c:spPr>
         </c:hiLowLines>
         <c:marker val="0"/>
-        <c:axId val="40988600"/>
-        <c:axId val="88148885"/>
+        <c:axId val="2339691"/>
+        <c:axId val="92619117"/>
       </c:lineChart>
       <c:catAx>
-        <c:axId val="40988600"/>
+        <c:axId val="2339691"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -1680,7 +1680,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="88148885"/>
+        <c:crossAx val="92619117"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -1688,7 +1688,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="88148885"/>
+        <c:axId val="92619117"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -1764,7 +1764,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="40988600"/>
+        <c:crossAx val="2339691"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -2121,11 +2121,11 @@
           </c:spPr>
         </c:hiLowLines>
         <c:marker val="0"/>
-        <c:axId val="20188616"/>
-        <c:axId val="1618004"/>
+        <c:axId val="65908982"/>
+        <c:axId val="75281032"/>
       </c:lineChart>
       <c:catAx>
-        <c:axId val="20188616"/>
+        <c:axId val="65908982"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -2191,7 +2191,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="1618004"/>
+        <c:crossAx val="75281032"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -2199,7 +2199,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="1618004"/>
+        <c:axId val="75281032"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -2275,7 +2275,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="20188616"/>
+        <c:crossAx val="65908982"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>

</xml_diff>